<commit_message>
P0: ferramenta de recuperação sem Get-FileHash (SHA-256 .NET); testes da desinstalação e do verificar corrigidos
CI 40979557950 (ad7434d): 41 aprovados, 6 reprovados. 2.10 (banco derrubado) aprovado: correção do syslogger
confirmada. Reprovações: Get-FileHash indisponível quando o PSModulePath vem do PowerShell 7 (Recuperar_VYONIX
usa agora SHA-256 do .NET; o CI chama o powershell.exe com os módulos do Windows PowerShell 5.1) e 3 em cascata;
log do Inno é ANSI (teste lia como UTF-8); verificar na porta movida pelo 2.7.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014XqvwZWSWShUuqoong32i9
</commit_message>
<xml_diff>
--- a/docs/homologacao/VYONIX_P0_Acompanhamento.xlsx
+++ b/docs/homologacao/VYONIX_P0_Acompanhamento.xlsx
@@ -22,9 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="90">
-  <si>
-    <t xml:space="preserve">VYONIX — P0: requisitos e situação (atualizado em 2026-10-29 21:40)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="94">
+  <si>
+    <t xml:space="preserve">VYONIX — P0: requisitos e situação (atualizado em 2026-10-29 22:45)</t>
   </si>
   <si>
     <t xml:space="preserve">Commit da implementação: ad7434d (P0) · c725108 (segurança) (ramo develop). Teste local ≠ CI Windows ≠ validação no computador do proprietário. Nada é marcado como aprovado sem execução. Células amarelas: atualizar.</t>
@@ -63,21 +63,24 @@
     <t xml:space="preserve">Aprovado</t>
   </si>
   <si>
+    <t xml:space="preserve">Pendente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI 2.12 run 40979557950: status final 'concluida' gravado e conferido após o término; reinstalar e atualizar com assistente aberto aprovados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove somente serviços do VYONIX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instalador e DEPLOY só tocam um serviço se o programa dele está em Program Files\VYONIX\Platform; serviço alheio com o mesmo nome nunca é alterado; DICOM Print nunca está na lista</t>
+  </si>
+  <si>
     <t xml:space="preserve">Não executado</t>
   </si>
   <si>
-    <t xml:space="preserve">Pendente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tests_deploy/test_uninstall.py::test_uninstaller_itself_is_never_killed; CI 2.12 (a executar)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remove somente serviços do VYONIX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Instalador e DEPLOY só tocam um serviço se o programa dele está em Program Files\VYONIX\Platform; serviço alheio com o mesmo nome nunca é alterado; DICOM Print nunca está na lista</t>
-  </si>
-  <si>
     <t xml:space="preserve">tests_deploy/test_uninstall.py::Ownership (3 testes); CI 2.13 serviço alheio (a executar)</t>
   </si>
   <si>
@@ -87,7 +90,7 @@
     <t xml:space="preserve">Verificação final do estado real (serviços, processos, pasta) em C:\ProgramData\VYONIX\Logs\desinstalacao.json (concluída / reiniciar / incompleta); 'incompleta' registra ERRO e mostra mensagem</t>
   </si>
   <si>
-    <t xml:space="preserve">test_inno_uninstaller_checks_ownership_and_final_state; CI 2.12 e homologação 15 (a executar)</t>
+    <t xml:space="preserve">test_inno_uninstaller_checks_ownership_and_final_state; CI 2.12 e homologação 15 (a executar); run 40979557950: status 'concluida' conferido; checagem do texto do log reprovou por codificação (teste corrigido)</t>
   </si>
   <si>
     <t xml:space="preserve">Testes sem condição de corrida</t>
@@ -117,7 +120,7 @@
     <t xml:space="preserve">Reversão de instalação com falha só remove banco/cluster comprovadamente criado na mesma execução; estado desconhecido nunca é removido</t>
   </si>
   <si>
-    <t xml:space="preserve">tests_deploy/test_faults.py (RollbackNeverDropsExistingDatabase, ClusterRollback); CI 2.13 falha na migração (a executar)</t>
+    <t xml:space="preserve">tests_deploy/test_faults.py (RollbackNeverDropsExistingDatabase, ClusterRollback); CI 2.13 falha na migração (a executar); CI 2.13 falha simulada na migração: rolled_back, banco preservado, restauração e nova atualização aprovadas (run 40979557950)</t>
   </si>
   <si>
     <t xml:space="preserve">Atualização sobre bc9cf28</t>
@@ -126,7 +129,7 @@
     <t xml:space="preserve">Homologação confere também migrações aplicadas, serviços e 'Verificar funcionamento'</t>
   </si>
   <si>
-    <t xml:space="preserve">Em b22bcc4: homologação 0a–15 aprovada (run 40951161126). Verificações ampliadas (migrações/serviços) rodam em ad7434d.</t>
+    <t xml:space="preserve">Homologação 0a–15 aprovada em ad7434d (run 40979622943)</t>
   </si>
   <si>
     <t xml:space="preserve">DICOM Print (testes que dependem de impressora/equipamento)</t>
@@ -144,7 +147,7 @@
     <t xml:space="preserve">Coletor de log do PostgreSQL desligado (registros no Log de Eventos); antes de iniciar o serviço parado, o DEPLOY encerra postgres.exe órfãos só da pasta do VYONIX; atualização reaplica a configuração</t>
   </si>
   <si>
-    <t xml:space="preserve">tests_deploy/test_faults.py::PostgresOrphans; causa no CI 40951093428 (syslogger com pai encerrado)</t>
+    <t xml:space="preserve">tests_deploy/test_faults.py::PostgresOrphans; causa no CI 40951093428 (syslogger com pai encerrado); CI 2.10 aprovado no run 40979557950 (ad7434d)</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo</t>
@@ -234,10 +237,7 @@
     <t xml:space="preserve">ad7434d</t>
   </si>
   <si>
-    <t xml:space="preserve">Em execução</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inclui a correção do banco (2.10), o desinstalador com verificação final e o critério 2.13</t>
+    <t xml:space="preserve">41 aprovados, 6 reprovados, 1 não executado (DICOM Print: impressora — registrado à parte). APROVADOS: 2.10 banco derrubado volta sozinho (correção do syslogger confirmada); reinstalar, atualizar por cima com assistente aberto, reparo; 2.13 diagnóstico só leitura, cancelamento, falha simulada na migração com restauração. REPROVADOS: ferramenta de recuperação (Get-FileHash indisponível com PSModulePath do PowerShell 7 → corrigido com SHA-256 .NET) e 3 em cascata; teste do registro da desinstalação lia o log ANSI como UTF-8 (teste); verificar na porta errada após 2.7 (teste).</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/well498/VYONIX-DICOMPRINT/actions/runs/40979557950</t>
@@ -246,10 +246,22 @@
     <t xml:space="preserve">40979622943</t>
   </si>
   <si>
-    <t xml:space="preserve">Inclui migrações/serviços/verificação após atualizar sobre bc9cf28 e a espera do fim real da desinstalação</t>
+    <t xml:space="preserve">Homologação 0a–15 aprovada em ad7434d (inclui verificação de migrações/serviços após atualizar sobre bc9cf28 e espera do fim real da desinstalação).</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/well498/VYONIX-DICOMPRINT/actions/runs/40979622943</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(a disparar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comercial + homologação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">próximo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correções da ferramenta de recuperação e dos testes; segurança c725108; botão da assinatura 76c6754</t>
   </si>
   <si>
     <t xml:space="preserve">Próximos passos</t>
@@ -773,15 +785,17 @@
         <v>12</v>
       </c>
       <c r="E5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="G5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="H5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
@@ -797,37 +811,37 @@
         <v>12</v>
       </c>
       <c r="E6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="G6" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="G7" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H7" s="5"/>
     </row>
@@ -836,22 +850,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="G8" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H8" s="5"/>
     </row>
@@ -860,98 +874,100 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>12</v>
       </c>
       <c r="E9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="G9" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>12</v>
       </c>
       <c r="E10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="G10" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="G11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H11" s="5"/>
+        <v>35</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="G12" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H12" s="5"/>
     </row>
@@ -960,36 +976,36 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>12</v>
       </c>
       <c r="E13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>14</v>
-      </c>
       <c r="G13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3" t="s">
@@ -999,7 +1015,7 @@
         <v>6</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1014,7 +1030,7 @@
       </c>
       <c r="E17" s="4" t="n">
         <f aca="false">COUNTIF(E$5:E$13,$B17)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F17" s="4" t="n">
         <f aca="false">COUNTIF(F$5:F$13,$B17)</f>
@@ -1024,7 +1040,7 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4"/>
       <c r="B18" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4" t="n">
@@ -1043,7 +1059,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4"/>
       <c r="B19" s="4" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4" t="n">
@@ -1052,7 +1068,7 @@
       </c>
       <c r="E19" s="4" t="n">
         <f aca="false">COUNTIF(E$5:E$13,$B19)</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F19" s="4" t="n">
         <f aca="false">COUNTIF(F$5:F$13,$B19)</f>
@@ -1062,7 +1078,7 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4" t="n">
@@ -1100,7 +1116,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -1114,136 +1130,136 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>8</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>71</v>
@@ -1251,20 +1267,22 @@
       <c r="F8" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G8" s="5"/>
+      <c r="G8" s="5" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
         <v>73</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>74</v>
@@ -1272,7 +1290,28 @@
       <c r="F9" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="5"/>
+      <c r="G9" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1307,7 +1346,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1315,13 +1354,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1329,13 +1368,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1343,13 +1382,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1357,13 +1396,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>86</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1371,18 +1410,18 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>